<commit_message>
Auto: Week 28/2026 data extracted from PDFs
</commit_message>
<xml_diff>
--- a/Gulf_Dashboard_W28_2026.xlsx
+++ b/Gulf_Dashboard_W28_2026.xlsx
@@ -729,30 +729,7 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>➢ 1.Delay of SAO bridge and box convert construction ( 3 bridges and 2 box culverts)
-➢ 2.Low production rate of rebar installation
-- WTG08 Rebar binding 66 Days
-- WTG06 Rebar binding 63 Days
-- WTG11 Rebar binding 39 Days
-- WTG12 Rebar binding 24 Days
-- WTG14 Rebar binding 26 Days
-Based on the current site arrangement, there is a drainage concern related to the Box Culvert area
-at East Side RW17 Sta 0+500, which may be affect to the equipment/material laydown arrangement
-from Silamas.
-Box culvert
-➢ 1.Request cooperation from Chief Executive of the
-Non sawang SAO incase stagnant water from road
-project. (Temporary protection completed,
-Permanent protection plan to start after WTG05
-➢ 2.Unofficial Environmental &amp; Social Complaints
-Local residents are complaining about stagnant water
-from road project
-- West side 2 person (Area same as first topic,RW5)
-- East side 6 person (RW17 STA 0+500)</t>
-        </is>
-      </c>
+      <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Backfilling
@@ -876,22 +853,7 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>requirements
-Material scrap storage and waste segregation were the most frequently
-observed findings this week. These issues were primarily attributed to the
-lack of waste segregation at the working area, insufficient provision of waste
-containers, and lack of clearly designated scrap storage areas.
-Lack of awarenessin waste management requirements contributed to these
-• At certain WTG locations, the Hardstand (TSA) level does not correspond with the road level (CBOP), which may have an
-adverse impact on the transportation and installation of the wind turbine components.
-• Grounding design is pending to be approved, which may impact to soil backfilling work after complete concrete curing
-period of WTG foundation.
-115kV Substation
-115kV Transmission Line</t>
-        </is>
-      </c>
+      <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr">
         <is>
           <t>➢ Continue to road base course compaction work.

</xml_diff>